<commit_message>
feat(sections): section-wise sorting, sectionIndex in API response, sections array in exam response, SMTP email results, negative marking, section-isolated shuffling
</commit_message>
<xml_diff>
--- a/bulk_import_template.xlsx
+++ b/bulk_import_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="54">
   <si>
     <t>Question Text *</t>
   </si>
@@ -41,6 +41,9 @@
     <t>Difficulty</t>
   </si>
   <si>
+    <t>Section Name</t>
+  </si>
+  <si>
     <t>What is the capital of India?</t>
   </si>
   <si>
@@ -62,6 +65,9 @@
     <t>easy</t>
   </si>
   <si>
+    <t>General</t>
+  </si>
+  <si>
     <t>Which of the following are programming languages?</t>
   </si>
   <si>
@@ -98,6 +104,9 @@
     <t>True</t>
   </si>
   <si>
+    <t>GK</t>
+  </si>
+  <si>
     <t>The speed of light is ___ km/s.</t>
   </si>
   <si>
@@ -110,6 +119,9 @@
     <t>hard</t>
   </si>
   <si>
+    <t>Physics</t>
+  </si>
+  <si>
     <t>What is 2 + 2?</t>
   </si>
   <si>
@@ -117,6 +129,9 @@
   </si>
   <si>
     <t>4</t>
+  </si>
+  <si>
+    <t>Maths</t>
   </si>
   <si>
     <t>BULK IMPORT TEMPLATE — INSTRUCTIONS</t>
@@ -158,6 +173,9 @@
   </si>
   <si>
     <t>One of: easy, medium, hard. Default: medium</t>
+  </si>
+  <si>
+    <t>Name of the section this question belongs to (e.g., "XYZ topic", "ABC topic"). Default: General</t>
   </si>
 </sst>
 </file>
@@ -574,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -583,9 +601,10 @@
     <col min="7" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -613,150 +632,168 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="H2" s="2">
         <v>2</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H3" s="3">
         <v>3</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H4" s="2">
         <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H5" s="3">
         <v>2</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H6" s="2">
         <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -767,7 +804,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -776,55 +813,55 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -832,7 +869,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -840,7 +877,15 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>